<commit_message>
update: cleaning and add contacts info
</commit_message>
<xml_diff>
--- a/Controle_Linhas_Aparelhos.xlsx
+++ b/Controle_Linhas_Aparelhos.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\suporte\Desktop\whatsapp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{0254497C-1627-49D2-9832-BF059C9912DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64113A95-EDF5-489B-BAF3-81C20FD616F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="20730" windowHeight="11760" xr2:uid="{98DFD1DF-0CCD-46B4-8C97-BAAFD7B9157E}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{98DFD1DF-0CCD-46B4-8C97-BAAFD7B9157E}"/>
   </bookViews>
   <sheets>
     <sheet name="devices_and_lines" sheetId="1" r:id="rId1"/>
+    <sheet name="contacts" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="39">
   <si>
     <t>device_name</t>
   </si>
@@ -132,6 +133,30 @@
   </si>
   <si>
     <t>LIVRE</t>
+  </si>
+  <si>
+    <t>Nome</t>
+  </si>
+  <si>
+    <t>eMail</t>
+  </si>
+  <si>
+    <t>joao.gollucci@gauge.haus</t>
+  </si>
+  <si>
+    <t>eduardo.lima@gauge.haus</t>
+  </si>
+  <si>
+    <t>João Gollucci</t>
+  </si>
+  <si>
+    <t>Eduardo Lima</t>
+  </si>
+  <si>
+    <t>Rafael Santana</t>
+  </si>
+  <si>
+    <t>prsantana2@gauge.haus</t>
   </si>
 </sst>
 </file>
@@ -213,6 +238,17 @@
     <tableColumn id="4" xr3:uid="{AAD6B6BA-5597-4570-AA95-2ED1F64CB6DC}" name="status"/>
     <tableColumn id="5" xr3:uid="{C354A769-BA92-4D96-A5BD-1EFA2F9B27F2}" name="app_link" dataCellStyle="Hiperlink"/>
     <tableColumn id="6" xr3:uid="{0C03088D-758B-4CF9-BECD-E471D91DC8FE}" name="db_folder"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{49DA2F92-970F-412E-B586-8C941347BE1A}" name="Tabela2" displayName="Tabela2" ref="A1:B4" totalsRowShown="0">
+  <autoFilter ref="A1:B4" xr:uid="{49DA2F92-970F-412E-B586-8C941347BE1A}"/>
+  <tableColumns count="2">
+    <tableColumn id="1" xr3:uid="{429879BE-4130-4731-9784-75C17BAC5E25}" name="Nome"/>
+    <tableColumn id="2" xr3:uid="{C253909C-64E7-40B3-8A48-4B54A3F2DE91}" name="eMail"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -673,4 +709,53 @@
     <tablePart r:id="rId5"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FAF64E35-DB6F-4059-86BD-EF7EE3B4B901}">
+  <dimension ref="A1:B4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="19.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="25" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>31</v>
+      </c>
+      <c r="B1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B2" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>36</v>
+      </c>
+      <c r="B3" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>37</v>
+      </c>
+      <c r="B4" t="s">
+        <v>38</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
 </file>
</xml_diff>